<commit_message>
docs: Review 2 test documents and Design Brief follow the dashboards of 30/10
- TC-RPT-015 (money and residents on the Manager and Admin dashboards, A-63)
  is a rule case of F-18; 169 designed cases, 149 automated; mvn verify on
  30/10/2026: 245 tests, 245 passed. Report 5 and the workbooks rebuilt.
- Design Brief: F-18 acceptance names the same money on every dashboard and
  no 100 % rate with debt left.
- Project Tracking: the two dashboard defects fixed on 30/10/2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reports/out/SWP490_FA26SE260_R2_ProjectTracking.xlsx
+++ b/docs/reports/out/SWP490_FA26SE260_R2_ProjectTracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\Project\CampusStay FPT\docs\reports\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD214528-B374-40F6-A03B-2B8B8B54989F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{49A8EDF8-F649-49D1-A716-B8EEDD9BAF4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="322">
   <si>
     <t>Notes</t>
   </si>
@@ -920,6 +920,21 @@
   </si>
   <si>
     <t>fix 28/10/2026: XLSX templates (commit 4138397)</t>
+  </si>
+  <si>
+    <t>Manager and Admin dashboards</t>
+  </si>
+  <si>
+    <t>Money collected differed between the dashboards and Collections and refunds (Deposits without a Bed left out); a rate with debt left could read 100 %</t>
+  </si>
+  <si>
+    <t>fix 30/10/2026 (A-63); TC-RPT-015</t>
+  </si>
+  <si>
+    <t>Admin dashboard</t>
+  </si>
+  <si>
+    <t>Residents counted only desk check-ins, not released door codes (ADR-23)</t>
   </si>
   <si>
     <t>Web screen map</t>
@@ -3672,7 +3687,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.44140625" customWidth="1"/>
@@ -4101,7 +4116,7 @@
     </row>
     <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="B21" s="20" t="s">
         <v>294</v>
@@ -4124,7 +4139,7 @@
     </row>
     <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="B22" s="20" t="s">
         <v>297</v>
@@ -4136,13 +4151,59 @@
         <v>298</v>
       </c>
       <c r="E22" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="G22" s="20" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>299</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="G23" s="20" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="E24" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="F22" s="20" t="s">
+      <c r="F24" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="20" t="s">
-        <v>299</v>
+      <c r="G24" s="20" t="s">
+        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -4195,10 +4256,10 @@
         <v>207</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>205</v>
@@ -4207,7 +4268,7 @@
         <v>209</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27" x14ac:dyDescent="0.3">
@@ -4215,10 +4276,10 @@
         <v>207</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>205</v>
@@ -4227,7 +4288,7 @@
         <v>209</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27" x14ac:dyDescent="0.3">
@@ -4235,10 +4296,10 @@
         <v>223</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>205</v>
@@ -4247,7 +4308,7 @@
         <v>209</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="27" x14ac:dyDescent="0.3">
@@ -4255,10 +4316,10 @@
         <v>219</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>205</v>
@@ -4267,7 +4328,7 @@
         <v>209</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="27" x14ac:dyDescent="0.3">
@@ -4275,10 +4336,10 @@
         <v>232</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>3</v>
@@ -4287,7 +4348,7 @@
         <v>20</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.3">
@@ -4295,10 +4356,10 @@
         <v>232</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>3</v>
@@ -4307,7 +4368,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="40.200000000000003" x14ac:dyDescent="0.3">
@@ -4315,10 +4376,10 @@
         <v>232</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>3</v>

</xml_diff>